<commit_message>
paper run 2026-09-21 11:56
</commit_message>
<xml_diff>
--- a/reports/2026-09-21.xlsx
+++ b/reports/2026-09-21.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,92 @@
       </c>
       <c r="K3" t="n">
         <v>57.59</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-21T08:54:10.287313+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F4" t="n">
+        <v>65.27</v>
+      </c>
+      <c r="G4" t="n">
+        <v>123.15</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.785</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00117</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>57.88</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-21T10:41:52.773202+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="G5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.775</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00124</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>5.52</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +679,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +689,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -623,7 +709,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +719,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23.67</v>
+        <v>87.06999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +729,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>57.59</v>
+        <v>120.99</v>
       </c>
     </row>
     <row r="8">
@@ -663,7 +749,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.7</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +759,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1305.42</v>
+        <v>1368.82</v>
       </c>
     </row>
     <row r="12">
@@ -724,16 +810,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>91.86</v>
+        <v>125.33</v>
       </c>
       <c r="E15" t="n">
-        <v>23.67</v>
+        <v>29.19</v>
       </c>
     </row>
     <row r="16">
@@ -743,16 +829,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>-62.39</v>
+        <v>39.78</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>57.88</v>
       </c>
     </row>
     <row r="17">
@@ -765,55 +851,55 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>-6.5</v>
+        <v>57.88</v>
       </c>
       <c r="E18" t="n">
-        <v>23.67</v>
+        <v>57.88</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>98.36</v>
+        <v>37.08</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>23.67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>-62.39</v>
+        <v>30.19</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -822,59 +908,71 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>39.96</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5.52</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-68.89</v>
-      </c>
-      <c r="E22" t="n">
-        <v>23.67</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>98.36</v>
+        <v>47.05</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>87.06999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>74.48</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -884,7 +982,7 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>47.07</v>
+        <v>43.58</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -893,112 +991,116 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>2</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="n">
-        <v>-11.1</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
         <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>-6.5</v>
+        <v>47.07</v>
       </c>
       <c r="E27" t="n">
-        <v>23.67</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="E29" t="n">
+        <v>87.06999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>ETH</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>23.67</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>57.88</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1011,124 +1113,134 @@
         <v>23.67</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>5.52</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="n">
-        <v>-33.92</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>57.59</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>29.19</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>57.88</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>23.67</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-33.92</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>57.59</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1138,29 +1250,29 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>57.59</v>
+        <v>57.88</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>-33.92</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1182,17 +1294,125 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>87.06999999999999</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="n">
+        <v>115.47</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-28.4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
         <v>2</v>
       </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" t="n">
-        <v>23.67</v>
+      <c r="D56" t="n">
+        <v>29.19</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>57.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-21 17:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-21.xlsx
+++ b/reports/2026-09-21.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,49 @@
       </c>
       <c r="K5" t="n">
         <v>5.52</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-21T14:13:46.612327+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.00106</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>-10.6</v>
       </c>
     </row>
   </sheetData>
@@ -657,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,7 +722,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -699,7 +742,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -709,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
@@ -719,7 +762,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87.06999999999999</v>
+        <v>76.47</v>
       </c>
     </row>
     <row r="7">
@@ -739,7 +782,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-33.92</v>
+        <v>-44.52</v>
       </c>
     </row>
     <row r="9">
@@ -749,7 +792,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3.57</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="10">
@@ -759,7 +802,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1368.82</v>
+        <v>1358.22</v>
       </c>
     </row>
     <row r="12">
@@ -810,13 +853,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>125.33</v>
+        <v>267.07</v>
       </c>
       <c r="E15" t="n">
         <v>29.19</v>
@@ -829,16 +872,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>39.78</v>
+        <v>80.81999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>57.88</v>
+        <v>47.28</v>
       </c>
     </row>
     <row r="17">
@@ -874,13 +917,13 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" t="n">
         <v>3</v>
       </c>
-      <c r="C19" t="n">
-        <v>2</v>
-      </c>
       <c r="D19" t="n">
-        <v>37.08</v>
+        <v>71.3</v>
       </c>
       <c r="E19" t="n">
         <v>23.67</v>
@@ -893,16 +936,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>30.19</v>
+        <v>-6.89</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>-10.6</v>
       </c>
     </row>
     <row r="21">
@@ -912,13 +955,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D21" t="n">
-        <v>39.96</v>
+        <v>225.6</v>
       </c>
       <c r="E21" t="n">
         <v>5.52</v>
@@ -938,16 +981,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>47.05</v>
+        <v>41.83</v>
       </c>
       <c r="E23" t="n">
-        <v>87.06999999999999</v>
+        <v>76.47</v>
       </c>
     </row>
     <row r="24">
@@ -957,13 +1000,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D24" t="n">
-        <v>74.48</v>
+        <v>211.65</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -976,13 +1019,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>43.58</v>
+        <v>94.41</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -1021,13 +1064,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D28" t="n">
-        <v>8.6</v>
+        <v>259.29</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1040,16 +1083,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C29" t="n">
         <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>109.44</v>
+        <v>41.53</v>
       </c>
       <c r="E29" t="n">
-        <v>87.06999999999999</v>
+        <v>76.47</v>
       </c>
     </row>
     <row r="31">
@@ -1116,131 +1159,131 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-10.6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>XRP</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
         <v>5.52</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>3</v>
-      </c>
-      <c r="C39" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" t="n">
-        <v>29.19</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="n">
+        <v>29.19</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>57.88</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>47.28</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" t="n">
-        <v>-33.92</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>57.59</v>
+        <v>-33.92</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1250,168 +1293,200 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>57.88</v>
+        <v>57.59</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>57.88</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" t="n">
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
         <v>5.52</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-10.6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>4</v>
-      </c>
-      <c r="C49" t="n">
-        <v>3</v>
-      </c>
-      <c r="D49" t="n">
-        <v>87.06999999999999</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>2</v>
-      </c>
-      <c r="C52" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" t="n">
-        <v>115.47</v>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>76.47</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="n">
         <v>2</v>
       </c>
-      <c r="C53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" t="n">
-        <v>-28.4</v>
+      <c r="D54" t="n">
+        <v>104.87</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>3</v>
-      </c>
-      <c r="C56" t="n">
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
         <v>2</v>
       </c>
-      <c r="D56" t="n">
-        <v>29.19</v>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>-28.4</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>18.59</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B57" t="n">
-        <v>1</v>
-      </c>
-      <c r="C57" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" t="n">
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
         <v>57.88</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-09-21 23:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-21.xlsx
+++ b/reports/2026-09-21.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,6 +687,49 @@
       </c>
       <c r="K6" t="n">
         <v>-10.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-21T18:33:52.175443+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F7" t="n">
+        <v>50.01</v>
+      </c>
+      <c r="G7" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.00109</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>46.16</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,7 +765,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -732,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -752,7 +795,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="6">
@@ -762,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>76.47</v>
+        <v>122.63</v>
       </c>
     </row>
     <row r="7">
@@ -772,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>120.99</v>
+        <v>167.15</v>
       </c>
     </row>
     <row r="8">
@@ -792,7 +835,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.72</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="10">
@@ -802,7 +845,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1358.22</v>
+        <v>1404.38</v>
       </c>
     </row>
     <row r="12">
@@ -853,13 +896,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D15" t="n">
-        <v>267.07</v>
+        <v>447.73</v>
       </c>
       <c r="E15" t="n">
         <v>29.19</v>
@@ -872,16 +915,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>80.81999999999999</v>
+        <v>256.23</v>
       </c>
       <c r="E16" t="n">
-        <v>47.28</v>
+        <v>93.44</v>
       </c>
     </row>
     <row r="17">
@@ -898,13 +941,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>57.88</v>
+        <v>128.1</v>
       </c>
       <c r="E18" t="n">
         <v>57.88</v>
@@ -917,16 +960,16 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="n">
         <v>4</v>
       </c>
-      <c r="C19" t="n">
-        <v>3</v>
-      </c>
       <c r="D19" t="n">
-        <v>71.3</v>
+        <v>133.99</v>
       </c>
       <c r="E19" t="n">
-        <v>23.67</v>
+        <v>69.83</v>
       </c>
     </row>
     <row r="20">
@@ -936,13 +979,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>-6.89</v>
+        <v>53.33</v>
       </c>
       <c r="E20" t="n">
         <v>-10.6</v>
@@ -955,13 +998,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C21" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D21" t="n">
-        <v>225.6</v>
+        <v>388.54</v>
       </c>
       <c r="E21" t="n">
         <v>5.52</v>
@@ -981,16 +1024,16 @@
         </is>
       </c>
       <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
         <v>7</v>
       </c>
-      <c r="C23" t="n">
-        <v>4</v>
-      </c>
       <c r="D23" t="n">
-        <v>41.83</v>
+        <v>234.96</v>
       </c>
       <c r="E23" t="n">
-        <v>76.47</v>
+        <v>122.63</v>
       </c>
     </row>
     <row r="24">
@@ -1000,13 +1043,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D24" t="n">
-        <v>211.65</v>
+        <v>302.95</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1019,13 +1062,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D25" t="n">
-        <v>94.41</v>
+        <v>166.05</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -1064,13 +1107,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C28" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>259.29</v>
+        <v>552.67</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1083,16 +1126,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>41.53</v>
+        <v>104.22</v>
       </c>
       <c r="E29" t="n">
-        <v>76.47</v>
+        <v>122.63</v>
       </c>
     </row>
     <row r="31">
@@ -1147,13 +1190,13 @@
         </is>
       </c>
       <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="n">
         <v>2</v>
       </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
       <c r="D35" t="n">
-        <v>23.67</v>
+        <v>69.83</v>
       </c>
     </row>
     <row r="36">
@@ -1233,13 +1276,13 @@
         </is>
       </c>
       <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" t="n">
         <v>2</v>
       </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
       <c r="D41" t="n">
-        <v>47.28</v>
+        <v>93.44</v>
       </c>
     </row>
     <row r="43">
@@ -1344,149 +1387,165 @@
         <v>-10.6</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>46.16</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>0.50–0.55</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>5</v>
-      </c>
-      <c r="C51" t="n">
-        <v>3</v>
-      </c>
-      <c r="D51" t="n">
-        <v>76.47</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B52" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>122.63</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>3</v>
-      </c>
-      <c r="C54" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" t="n">
-        <v>104.87</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" t="n">
+        <v>3</v>
+      </c>
+      <c r="D55" t="n">
+        <v>151.03</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>0.12–0.15%</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B56" t="n">
         <v>2</v>
       </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="n">
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
         <v>-28.4</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>4</v>
-      </c>
-      <c r="C58" t="n">
-        <v>2</v>
-      </c>
-      <c r="D58" t="n">
-        <v>18.59</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>5</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>64.75</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B59" t="n">
-        <v>1</v>
-      </c>
-      <c r="C59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" t="n">
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
         <v>57.88</v>
       </c>
     </row>

</xml_diff>